<commit_message>
update xy2662 solo pipeline failure case
</commit_message>
<xml_diff>
--- a/result_data/xy2662.xlsx
+++ b/result_data/xy2662.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="result" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,13 +416,13 @@
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
@@ -507,7 +507,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>产物不满意：核心产物偏离提示词，后端入口、README 和测试脚本均实现手机维修工单流程，npm test 也只验证 /api/orders 的报价、维修、取机状态，未实现摄影棚位预约、押金核销/退款审计等要求。</t>
+          <t>产物不满意：核心 CSV 导出流程未跑通，/api/csv/export 和 /api/csv/all 均因中文 Content-Disposition 文件名触发 500，无法按提示词导出当天核销报表。</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>